<commit_message>
Build estate022 real parcel bbox final outputs
</commit_message>
<xml_diff>
--- a/ai-results/TerraYield_Emlakci_Parsel_Eslesme_FINAL.xlsx
+++ b/ai-results/TerraYield_Emlakci_Parsel_Eslesme_FINAL.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AAYS_GITHUB_BRIDGE_CLEAN2\ai-results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{372944AE-77E9-437D-A6AB-055C800C15CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{761F14A6-6AF6-467F-BEC2-16BE77423B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2618ACBC-B2C1-4713-AB30-F85B1300649F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7AA7A21F-28D4-4842-AB3C-63544B8A9944}"/>
   </bookViews>
   <sheets>
-    <sheet name="Real100_Status" sheetId="1" r:id="rId1"/>
+    <sheet name="Final_Status" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,10 +47,10 @@
     <t>value</t>
   </si>
   <si>
-    <t>verified_candidate_rows</t>
-  </si>
-  <si>
-    <t>parcel_candidate_files</t>
+    <t>parcel_join_rows</t>
+  </si>
+  <si>
+    <t>coverage_rows</t>
   </si>
   <si>
     <t>db_write</t>
@@ -59,10 +59,10 @@
     <t>production_deploy</t>
   </si>
   <si>
-    <t>final_status</t>
-  </si>
-  <si>
-    <t>review_required_not_import_ready</t>
+    <t>real_100</t>
+  </si>
+  <si>
+    <t>false_until_approval</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D74B5F-9E5B-4B9F-89C6-CAC160A6E993}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF47F19-893E-4654-93AF-50950DC34430}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -451,7 +451,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -459,7 +459,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>359</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>